<commit_message>
Correction chemin et ajout livrable
reste à relire, corriger le css sur certaines images et rajouter la video et les balise download pour livrables
</commit_message>
<xml_diff>
--- a/Le cabinet/Le_cabinet/livrables/num-plan.xlsx
+++ b/Le cabinet/Le_cabinet/livrables/num-plan.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
   <si>
     <t>Rôle</t>
   </si>
@@ -81,6 +81,20 @@
   </si>
   <si>
     <t>*1</t>
+  </si>
+  <si>
+    <t>Boîte Vocale</t>
+  </si>
+  <si>
+    <t>8500
+Identifiant: 
+Kiné Julien : 251
+Kiné Lisa -Marie : 252
+Kiné Clement : 253
+Dr Victor : 254
+Dr Angelo : 255
+Secrétaire : 256
+Mot de pass : 0000</t>
   </si>
 </sst>
 </file>
@@ -146,7 +160,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -158,6 +172,9 @@
     </xf>
     <xf borderId="1" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -492,6 +509,14 @@
         <v>22</v>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>24</v>
+      </c>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>